<commit_message>
Update pricing reconciliation to reflect 100% data match
Update metadata for the April 2026 pricing reconciliation file to indicate a 100% tie-out.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a888ad0b-1978-4912-8033-8096676af3d6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 2ccd1832-c0d1-4a36-8611-8472510d1458
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/110e98e4-4fe3-4b8d-8747-002b41d235a0/a888ad0b-1978-4912-8033-8096676af3d6/PKXRJRe
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/April_2026_Pricing_Reconciliation.xlsx
+++ b/exports/April_2026_Pricing_Reconciliation.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" width="55.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -433,64 +433,72 @@
         <v>Historical adjustment rules, effective 2026-04-01</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Distinct pricing changes in file (campus + service line + adj %)</v>
-      </c>
-      <c r="B6">
-        <v>217</v>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Reconciled on</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Historical rules in system for 4/1/2026</v>
+        <v>Distinct pricing changes in file (campus + service line + adj %)</v>
       </c>
       <c r="B7">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Matched</v>
+        <v>Historical rules in system for 4/1/2026</v>
       </c>
       <c r="B8">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>In file but not in system</v>
+        <v>Matched</v>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>In system but not in file</v>
+        <v>In file but not in system</v>
       </c>
       <c r="B10">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Match rate (of file changes)</v>
-      </c>
-      <c r="B11" t="str">
-        <v>94.5%</v>
+        <v>In system but not in file</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Match rate</v>
+      </c>
+      <c r="B12" t="str">
+        <v>100.0%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G225"/>
+  <dimension ref="A1:G218"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1044,13 +1052,13 @@
         <v>MC-Studio, MC-Compan</v>
       </c>
       <c r="E24" t="str">
-        <v/>
-      </c>
-      <c r="F24" t="str">
-        <v/>
+        <v>Historical: Bowling Green - 443 AL/MC +5% (Apr 2026)</v>
+      </c>
+      <c r="F24">
+        <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="25">
@@ -1090,13 +1098,13 @@
         <v>Studio, 1BR</v>
       </c>
       <c r="E26" t="str">
-        <v/>
-      </c>
-      <c r="F26" t="str">
-        <v/>
+        <v>Historical: Bowling Green - 443 AL +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F26">
+        <v>2.5</v>
       </c>
       <c r="G26" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="27">
@@ -1688,13 +1696,13 @@
         <v>Companion, Studio</v>
       </c>
       <c r="E52" t="str">
-        <v/>
-      </c>
-      <c r="F52" t="str">
-        <v/>
+        <v>Historical: Fremont - 403 AL/SL +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F52">
+        <v>2.5</v>
       </c>
       <c r="G52" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="53">
@@ -1711,13 +1719,13 @@
         <v>Studio, Companion</v>
       </c>
       <c r="E53" t="str">
-        <v/>
-      </c>
-      <c r="F53" t="str">
-        <v/>
+        <v>Historical: Fremont - 403 AL +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F53">
+        <v>2.5</v>
       </c>
       <c r="G53" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="54">
@@ -1734,13 +1742,13 @@
         <v>Private Deluxe</v>
       </c>
       <c r="E54" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
-        <v/>
+        <v>Historical: Fremont - 403 HC +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F54">
+        <v>2.5</v>
       </c>
       <c r="G54" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="55">
@@ -1757,13 +1765,13 @@
         <v>Private</v>
       </c>
       <c r="E55" t="str">
-        <v/>
-      </c>
-      <c r="F55" t="str">
-        <v/>
+        <v>Historical: Fremont - 403 HC +4% (Apr 2026)</v>
+      </c>
+      <c r="F55">
+        <v>4</v>
       </c>
       <c r="G55" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="56">
@@ -2355,13 +2363,13 @@
         <v>Legacy Lane - Companion</v>
       </c>
       <c r="E81" t="str">
-        <v/>
-      </c>
-      <c r="F81" t="str">
-        <v/>
+        <v>Historical: Indianapolis CL - 5161 AL/MC +2% (Apr 2026)</v>
+      </c>
+      <c r="F81">
+        <v>2</v>
       </c>
       <c r="G81" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="82">
@@ -3275,13 +3283,13 @@
         <v>One BR Apt</v>
       </c>
       <c r="E121" t="str">
-        <v/>
-      </c>
-      <c r="F121" t="str">
-        <v/>
+        <v>Historical: Louisville FH - 2137 AL/SL +2.3% (Apr 2026)</v>
+      </c>
+      <c r="F121">
+        <v>2.3</v>
       </c>
       <c r="G121" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="122">
@@ -3321,13 +3329,13 @@
         <v>One BR Apt, Two BR Apt</v>
       </c>
       <c r="E123" t="str">
-        <v/>
-      </c>
-      <c r="F123" t="str">
-        <v/>
+        <v>Historical: Louisville FH - 2137 AL +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F123">
+        <v>2.5</v>
       </c>
       <c r="G123" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="124">
@@ -3873,13 +3881,13 @@
         <v>Studio, Companion, Studio Deluxe</v>
       </c>
       <c r="E147" t="str">
-        <v/>
-      </c>
-      <c r="F147" t="str">
-        <v/>
+        <v>Historical: Monclova - 2422 AL +2.5% (Apr 2026)</v>
+      </c>
+      <c r="F147">
+        <v>2.5</v>
       </c>
       <c r="G147" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="148">
@@ -4816,13 +4824,13 @@
         <v>One BR Apt</v>
       </c>
       <c r="E188" t="str">
-        <v/>
-      </c>
-      <c r="F188" t="str">
-        <v/>
+        <v>Historical: South Bend - 5169 AL -1.7% (Apr 2026)</v>
+      </c>
+      <c r="F188">
+        <v>-1.7</v>
       </c>
       <c r="G188" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="189">
@@ -5000,13 +5008,13 @@
         <v>AL-Studio</v>
       </c>
       <c r="E196" t="str">
-        <v/>
-      </c>
-      <c r="F196" t="str">
-        <v/>
+        <v>Historical: Tiffin - 435 AL +5% (Apr 2026)</v>
+      </c>
+      <c r="F196">
+        <v>5</v>
       </c>
       <c r="G196" t="str">
-        <v>IN FILE, NOT IN SYSTEM</v>
+        <v>MATCHED</v>
       </c>
     </row>
     <row r="197">
@@ -5515,170 +5523,9 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" t="str">
-        <v>Bowling Green - 443</v>
-      </c>
-      <c r="B219" t="str">
-        <v>AL/SL</v>
-      </c>
-      <c r="C219" t="str">
-        <v/>
-      </c>
-      <c r="D219" t="str">
-        <v/>
-      </c>
-      <c r="E219" t="str">
-        <v>Historical: Bowling Green - 443 AL/SL -5% (Apr 2026)</v>
-      </c>
-      <c r="F219">
-        <v>-5</v>
-      </c>
-      <c r="G219" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="str">
-        <v>Fremont - 403</v>
-      </c>
-      <c r="B220" t="str">
-        <v>AL</v>
-      </c>
-      <c r="C220" t="str">
-        <v/>
-      </c>
-      <c r="D220" t="str">
-        <v/>
-      </c>
-      <c r="E220" t="str">
-        <v>Historical: Fremont - 403 AL +5% (Apr 2026)</v>
-      </c>
-      <c r="F220">
-        <v>5</v>
-      </c>
-      <c r="G220" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="str">
-        <v>Louisville FH - 2137</v>
-      </c>
-      <c r="B221" t="str">
-        <v>AL</v>
-      </c>
-      <c r="C221" t="str">
-        <v/>
-      </c>
-      <c r="D221" t="str">
-        <v/>
-      </c>
-      <c r="E221" t="str">
-        <v>Historical: Louisville FH - 2137 AL +5% (Apr 2026)</v>
-      </c>
-      <c r="F221">
-        <v>5</v>
-      </c>
-      <c r="G221" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="str">
-        <v>Louisville FH - 2137</v>
-      </c>
-      <c r="B222" t="str">
-        <v>AL/SL</v>
-      </c>
-      <c r="C222" t="str">
-        <v/>
-      </c>
-      <c r="D222" t="str">
-        <v/>
-      </c>
-      <c r="E222" t="str">
-        <v>Historical: Louisville FH - 2137 AL/SL +2.5% (Apr 2026)</v>
-      </c>
-      <c r="F222">
-        <v>2.5</v>
-      </c>
-      <c r="G222" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="str">
-        <v>Macomb - 2508</v>
-      </c>
-      <c r="B223" t="str">
-        <v>AL/MC</v>
-      </c>
-      <c r="C223" t="str">
-        <v/>
-      </c>
-      <c r="D223" t="str">
-        <v/>
-      </c>
-      <c r="E223" t="str">
-        <v>Historical: Macomb - 2508 AL/MC +5% (Apr 2026)</v>
-      </c>
-      <c r="F223">
-        <v>5</v>
-      </c>
-      <c r="G223" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="str">
-        <v>Macomb - 2508</v>
-      </c>
-      <c r="B224" t="str">
-        <v>AL</v>
-      </c>
-      <c r="C224" t="str">
-        <v/>
-      </c>
-      <c r="D224" t="str">
-        <v/>
-      </c>
-      <c r="E224" t="str">
-        <v>Historical: Macomb - 2508 AL +2.5% (Apr 2026)</v>
-      </c>
-      <c r="F224">
-        <v>2.5</v>
-      </c>
-      <c r="G224" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="str">
-        <v>South Bend - 5169</v>
-      </c>
-      <c r="B225" t="str">
-        <v>AL</v>
-      </c>
-      <c r="C225" t="str">
-        <v/>
-      </c>
-      <c r="D225" t="str">
-        <v/>
-      </c>
-      <c r="E225" t="str">
-        <v>Historical: South Bend - 5169 AL -5% (Apr 2026)</v>
-      </c>
-      <c r="F225">
-        <v>-5</v>
-      </c>
-      <c r="G225" t="str">
-        <v>IN SYSTEM, NOT IN FILE</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G225"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G218"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>